<commit_message>
22127410: note in checklist
</commit_message>
<xml_diff>
--- a/project/HW4/22127310/22127310_GUI_Checklist.xlsx
+++ b/project/HW4/22127310/22127310_GUI_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thanhthuy/Documents/Testing-PRJ-SM/project/HW4/22127310/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7782281-6C6C-DC47-9C5B-755BC4747C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1F82692-D744-E949-9F46-D61A9AE6257D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GUI list" sheetId="2" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="168">
   <si>
     <t>ID</t>
   </si>
@@ -524,6 +524,15 @@
   </si>
   <si>
     <t>Trang web có tiêu đề rõ ràng không?</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>All pages</t>
+  </si>
+  <si>
+    <t>This page only</t>
   </si>
 </sst>
 </file>
@@ -592,7 +601,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -608,12 +617,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -719,10 +722,10 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
@@ -776,14 +779,15 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="A4:E86" totalsRowShown="0">
-  <autoFilter ref="A4:E86" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="A4:F86" totalsRowShown="0">
+  <autoFilter ref="A4:F86" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="No." dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Checkpoints" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Yes" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="No" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Remarks"/>
+    <tableColumn id="6" xr3:uid="{CE5C7A42-BE31-3046-BD5B-C4B9CADC712E}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1133,6 +1137,7 @@
     <col min="1" max="1" width="8.83203125" style="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="82" style="2" customWidth="1"/>
     <col min="3" max="4" width="6.33203125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -1145,6 +1150,7 @@
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
       <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="2" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
@@ -1156,6 +1162,7 @@
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
       <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
@@ -1165,7 +1172,7 @@
       <c r="C3" s="15"/>
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
-      <c r="F3" s="3"/>
+      <c r="F3" s="15"/>
       <c r="H3" s="3"/>
       <c r="I3" s="17"/>
     </row>
@@ -1185,6 +1192,9 @@
       <c r="E4" s="5" t="s">
         <v>116</v>
       </c>
+      <c r="F4" s="5" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="5" spans="1:9" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18">
@@ -1196,6 +1206,7 @@
       <c r="C5" s="20"/>
       <c r="D5" s="20"/>
       <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
     </row>
     <row r="6" spans="1:9" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18">
@@ -1207,6 +1218,7 @@
       <c r="C6" s="20"/>
       <c r="D6" s="20"/>
       <c r="E6" s="20"/>
+      <c r="F6" s="21"/>
     </row>
     <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
@@ -1218,6 +1230,9 @@
       <c r="C7" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F7" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="10" t="s">
@@ -1229,6 +1244,9 @@
       <c r="C8" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F8" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
@@ -1240,6 +1258,9 @@
       <c r="D9" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F9" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="26" t="s">
@@ -1251,6 +1272,9 @@
       <c r="D10" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F10" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="11" spans="1:9" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="19">
@@ -1262,6 +1286,7 @@
       <c r="C11" s="19"/>
       <c r="D11" s="19"/>
       <c r="E11" s="19"/>
+      <c r="F11" s="21"/>
     </row>
     <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
@@ -1273,6 +1298,9 @@
       <c r="D12" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F12" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
@@ -1284,6 +1312,9 @@
       <c r="D13" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F13" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
@@ -1295,6 +1326,9 @@
       <c r="C14" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F14" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
@@ -1306,6 +1340,9 @@
       <c r="C15" s="6" t="s">
         <v>138</v>
       </c>
+      <c r="F15" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
@@ -1317,8 +1354,11 @@
       <c r="C16" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
         <v>98</v>
       </c>
@@ -1328,8 +1368,11 @@
       <c r="C17" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
         <v>103</v>
       </c>
@@ -1339,8 +1382,11 @@
       <c r="C18" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F18" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
         <v>104</v>
       </c>
@@ -1350,8 +1396,11 @@
       <c r="C19" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="19">
         <v>1.3</v>
       </c>
@@ -1361,8 +1410,9 @@
       <c r="C20" s="19"/>
       <c r="D20" s="19"/>
       <c r="E20" s="19"/>
-    </row>
-    <row r="21" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="F20" s="21"/>
+    </row>
+    <row r="21" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
         <v>57</v>
       </c>
@@ -1372,8 +1422,11 @@
       <c r="C21" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F21" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
         <v>58</v>
       </c>
@@ -1383,8 +1436,11 @@
       <c r="C22" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F22" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
         <v>59</v>
       </c>
@@ -1394,8 +1450,11 @@
       <c r="C23" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F23" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
         <v>60</v>
       </c>
@@ -1405,8 +1464,11 @@
       <c r="C24" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F24" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
         <v>105</v>
       </c>
@@ -1416,8 +1478,11 @@
       <c r="D25" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F25" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
         <v>106</v>
       </c>
@@ -1427,8 +1492,11 @@
       <c r="C26" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
         <v>107</v>
       </c>
@@ -1438,8 +1506,11 @@
       <c r="C27" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F27" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
         <v>108</v>
       </c>
@@ -1449,8 +1520,11 @@
       <c r="C28" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F28" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="26" t="s">
         <v>109</v>
       </c>
@@ -1460,8 +1534,11 @@
       <c r="D29" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F29" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="26" t="s">
         <v>110</v>
       </c>
@@ -1471,8 +1548,11 @@
       <c r="C30" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F30" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="5" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="25" t="s">
         <v>139</v>
       </c>
@@ -1482,8 +1562,9 @@
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
       <c r="E31" s="19"/>
-    </row>
-    <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F31" s="21"/>
+    </row>
+    <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="24" t="s">
         <v>111</v>
       </c>
@@ -1491,7 +1572,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="27" t="s">
         <v>140</v>
       </c>
@@ -1501,8 +1582,11 @@
       <c r="C33" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F33" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="27" t="s">
         <v>141</v>
       </c>
@@ -1512,8 +1596,11 @@
       <c r="C34" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="F34" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="27" t="s">
         <v>142</v>
       </c>
@@ -1523,8 +1610,11 @@
       <c r="C35" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="F35" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="27" t="s">
         <v>143</v>
       </c>
@@ -1534,8 +1624,11 @@
       <c r="C36" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F36" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="27" t="s">
         <v>144</v>
       </c>
@@ -1545,8 +1638,11 @@
       <c r="C37" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" s="5" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F37" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="24" t="s">
         <v>112</v>
       </c>
@@ -1557,7 +1653,7 @@
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
     </row>
-    <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
         <v>155</v>
       </c>
@@ -1567,8 +1663,11 @@
       <c r="D39" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F39" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
         <v>156</v>
       </c>
@@ -1578,8 +1677,11 @@
       <c r="D40" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F40" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="10" t="s">
         <v>157</v>
       </c>
@@ -1589,8 +1691,11 @@
       <c r="D41" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F41" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
         <v>113</v>
       </c>
@@ -1598,7 +1703,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="26" t="s">
         <v>145</v>
       </c>
@@ -1608,8 +1713,11 @@
       <c r="D43" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F43" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="26" t="s">
         <v>146</v>
       </c>
@@ -1619,8 +1727,11 @@
       <c r="D44" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F44" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="26" t="s">
         <v>147</v>
       </c>
@@ -1631,8 +1742,11 @@
       <c r="D45" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F45" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="26" t="s">
         <v>148</v>
       </c>
@@ -1642,8 +1756,11 @@
       <c r="D46" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F46" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="26" t="s">
         <v>149</v>
       </c>
@@ -1653,8 +1770,11 @@
       <c r="C47" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F47" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="26" t="s">
         <v>150</v>
       </c>
@@ -1664,8 +1784,11 @@
       <c r="C48" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F48" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="26" t="s">
         <v>151</v>
       </c>
@@ -1675,8 +1798,11 @@
       <c r="C49" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F49" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="26" t="s">
         <v>152</v>
       </c>
@@ -1687,8 +1813,11 @@
         <v>138</v>
       </c>
       <c r="D50" s="8"/>
-    </row>
-    <row r="51" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F50" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="26" t="s">
         <v>153</v>
       </c>
@@ -1698,8 +1827,11 @@
       <c r="D51" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F51" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="26" t="s">
         <v>154</v>
       </c>
@@ -1709,8 +1841,11 @@
       <c r="C52" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F52" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="26" t="s">
         <v>162</v>
       </c>
@@ -1720,8 +1855,11 @@
       <c r="C53" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F53" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="18">
         <v>2</v>
       </c>
@@ -1731,8 +1869,9 @@
       <c r="C54" s="22"/>
       <c r="D54" s="22"/>
       <c r="E54" s="23"/>
-    </row>
-    <row r="55" spans="1:5" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F54" s="21"/>
+    </row>
+    <row r="55" spans="1:6" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="18">
         <v>2.1</v>
       </c>
@@ -1742,8 +1881,9 @@
       <c r="C55" s="22"/>
       <c r="D55" s="22"/>
       <c r="E55" s="22"/>
-    </row>
-    <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F55" s="21"/>
+    </row>
+    <row r="56" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="10" t="s">
         <v>61</v>
       </c>
@@ -1753,8 +1893,11 @@
       <c r="C56" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F56" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="10" t="s">
         <v>99</v>
       </c>
@@ -1764,8 +1907,11 @@
       <c r="C57" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F57" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="26" t="s">
         <v>100</v>
       </c>
@@ -1775,8 +1921,11 @@
       <c r="D58" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F58" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="10" t="s">
         <v>114</v>
       </c>
@@ -1786,8 +1935,11 @@
       <c r="D59" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F59" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="18">
         <v>2.2000000000000002</v>
       </c>
@@ -1797,8 +1949,9 @@
       <c r="C60" s="19"/>
       <c r="D60" s="19"/>
       <c r="E60" s="19"/>
-    </row>
-    <row r="61" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F60" s="21"/>
+    </row>
+    <row r="61" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="10" t="s">
         <v>62</v>
       </c>
@@ -1808,8 +1961,11 @@
       <c r="C61" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F61" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="10" t="s">
         <v>63</v>
       </c>
@@ -1819,8 +1975,11 @@
       <c r="C62" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F62" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="10" t="s">
         <v>120</v>
       </c>
@@ -1830,8 +1989,11 @@
       <c r="C63" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F63" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="10" t="s">
         <v>121</v>
       </c>
@@ -1841,8 +2003,11 @@
       <c r="C64" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F64" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="10" t="s">
         <v>122</v>
       </c>
@@ -1852,8 +2017,11 @@
       <c r="D65" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F65" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="10" t="s">
         <v>123</v>
       </c>
@@ -1863,8 +2031,11 @@
       <c r="C66" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F66" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="10" t="s">
         <v>124</v>
       </c>
@@ -1874,8 +2045,11 @@
       <c r="C67" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F67" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="10" t="s">
         <v>125</v>
       </c>
@@ -1885,8 +2059,11 @@
       <c r="C68" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F68" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="10" t="s">
         <v>126</v>
       </c>
@@ -1896,8 +2073,11 @@
       <c r="C69" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F69" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="10" t="s">
         <v>127</v>
       </c>
@@ -1907,8 +2087,11 @@
       <c r="D70" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F70" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="18">
         <v>3</v>
       </c>
@@ -1918,8 +2101,9 @@
       <c r="C71" s="19"/>
       <c r="D71" s="19"/>
       <c r="E71" s="19"/>
-    </row>
-    <row r="72" spans="1:5" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F71" s="21"/>
+    </row>
+    <row r="72" spans="1:6" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="18">
         <v>3.1</v>
       </c>
@@ -1929,8 +2113,9 @@
       <c r="C72" s="19"/>
       <c r="D72" s="19"/>
       <c r="E72" s="19"/>
-    </row>
-    <row r="73" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F72" s="21"/>
+    </row>
+    <row r="73" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A73" s="10" t="s">
         <v>65</v>
       </c>
@@ -1940,8 +2125,11 @@
       <c r="C73" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F73" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A74" s="10" t="s">
         <v>66</v>
       </c>
@@ -1951,8 +2139,11 @@
       <c r="D74" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F74" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A75" s="10" t="s">
         <v>84</v>
       </c>
@@ -1962,8 +2153,11 @@
       <c r="C75" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F75" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="10" t="s">
         <v>85</v>
       </c>
@@ -1973,8 +2167,11 @@
       <c r="C76" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="F76" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A77" s="10" t="s">
         <v>86</v>
       </c>
@@ -1984,8 +2181,11 @@
       <c r="C77" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F77" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="18">
         <v>3.2</v>
       </c>
@@ -1995,8 +2195,9 @@
       <c r="C78" s="19"/>
       <c r="D78" s="19"/>
       <c r="E78" s="19"/>
-    </row>
-    <row r="79" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="F78" s="21"/>
+    </row>
+    <row r="79" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A79" s="10" t="s">
         <v>69</v>
       </c>
@@ -2006,8 +2207,11 @@
       <c r="C79" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F79" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" s="10" t="s">
         <v>70</v>
       </c>
@@ -2017,8 +2221,11 @@
       <c r="C80" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F80" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" s="5" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="18">
         <v>3.3</v>
       </c>
@@ -2028,8 +2235,9 @@
       <c r="C81" s="19"/>
       <c r="D81" s="19"/>
       <c r="E81" s="19"/>
-    </row>
-    <row r="82" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F81" s="21"/>
+    </row>
+    <row r="82" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="10" t="s">
         <v>73</v>
       </c>
@@ -2039,8 +2247,11 @@
       <c r="C82" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F82" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="10" t="s">
         <v>74</v>
       </c>
@@ -2050,8 +2261,11 @@
       <c r="C83" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F83" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="10" t="s">
         <v>87</v>
       </c>
@@ -2061,8 +2275,11 @@
       <c r="D84" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F84" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A85" s="10" t="s">
         <v>88</v>
       </c>
@@ -2072,8 +2289,11 @@
       <c r="D85" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="F85" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" s="10" t="s">
         <v>89</v>
       </c>
@@ -2082,6 +2302,9 @@
       </c>
       <c r="C86" s="6" t="s">
         <v>138</v>
+      </c>
+      <c r="F86" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>